<commit_message>
Task 1: problem framing + channel-aware synthetic data generator
- src/cpg_forecast/data/: schema (pydantic + 15-col contract), reference master
  data (markets/brands/channels/packs), per-market holiday calendars, and a
  seeded DGP generator (trend, weekly+annual seasonality w/ hemisphere flip,
  holidays, promos+price elasticity, weather, intermittency, cold-start,
  stockout censoring, channel effects, Poisson noise); CLI + --sample
- tests: schema, determinism, no-NaN/negative, channel-in-market, hierarchy, promo
- docs/problem_spec.md; docs/Task1_Summary.xlsx (5 sheets)
- full dataset ~991K rows/960 series in ~3s, 1.4MB (git-ignored; DVC pending)
- gitignore data/synthetic/; statuses -> Task 1 done, Task 2 next
</commit_message>
<xml_diff>
--- a/docs/Roadmap.xlsx
+++ b/docs/Roadmap.xlsx
@@ -755,7 +755,7 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>1 done, 1 next, 17 planned</t>
+          <t>2 done, 1 next, 16 planned</t>
         </is>
       </c>
     </row>
@@ -953,9 +953,9 @@
           <t>Mac</t>
         </is>
       </c>
-      <c r="G4" s="8" t="inlineStr">
-        <is>
-          <t>Next</t>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -990,9 +990,9 @@
           <t>Mac</t>
         </is>
       </c>
-      <c r="G5" s="9" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>Next</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Task 2: EDA + fix two generator bugs found via EDA
- src/cpg_forecast/eda.py: reproducible EDA (findings + 7 figures), tested helpers
- FIX generator: hemisphere-aware annual seasonality (AU peaks in AU summer,
  weather corr +0.90 not -0.42); GT channel volume raised so Traditional Trade is
  dominant in India(52%)/Pakistan(65%)
- docs/eda_findings.md + docs/eda/*.png + docs/Task2_Summary.xlsx; tests/test_eda.py
- ruff isort known-first-party=cpg_forecast (stop pre-commit vs local ruff fights)
- make eda / task2-summary; DVC pointer updated; statuses -> Task 2 done, Task 3 next
</commit_message>
<xml_diff>
--- a/docs/Roadmap.xlsx
+++ b/docs/Roadmap.xlsx
@@ -755,7 +755,7 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>2 done, 1 next, 16 planned</t>
+          <t>3 done, 1 next, 15 planned</t>
         </is>
       </c>
     </row>
@@ -990,9 +990,9 @@
           <t>Mac</t>
         </is>
       </c>
-      <c r="G5" s="8" t="inlineStr">
-        <is>
-          <t>Next</t>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -1027,9 +1027,9 @@
           <t>Mac</t>
         </is>
       </c>
-      <c r="G6" s="9" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>Next</t>
         </is>
       </c>
     </row>

</xml_diff>